<commit_message>
Distribución: Drive limpio, proyecto actualizado, tarea semanal y ajustes finales
- Plan: punto de equilibrio con costos variables y fijos; referencia FOB por producto
  explicada; formato de porcentajes corregido; vida útil y tasas en el anexo.
- Resumen en inglés: presentaciones tal como están en el pliego de la LPU.
- DD y negociación: citas y redacción afinadas.
- Bitácora: estructura de Drive y del proyecto, tarea programada, cómo recrear
  private/; la auditoría avisa si falta la lista de nombres privados.
- README: dónde se distribuye cada documento y comprobación del Excel.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0135fezQES4kQref5cVQmNrQ
</commit_message>
<xml_diff>
--- a/outputs/Modelo_financiero.xlsx
+++ b/outputs/Modelo_financiero.xlsx
@@ -2103,7 +2103,7 @@
       </c>
       <c r="H29" s="15" t="inlineStr">
         <is>
-          <t>F: el pliego exige 18 meses de vida útil al entregar; con 24 meses de vida útil quedan unos 3 meses de ventana en bodega; E: frecuencia</t>
+          <t>F: el pliego pide el vencimiento de la ficha técnica o, si no lo fija, 18 meses de vida útil al entregar; con 24 meses de vida útil quedan unos 3 meses de ventana en bodega; E: frecuencia</t>
         </is>
       </c>
     </row>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="H32" s="15" t="inlineStr">
         <is>
-          <t>E: limitada por la vida útil (18 meses exigidos al entregar)</t>
+          <t>E: limitada por la vida útil exigida al entregar (18 meses si la ficha técnica no fija otra)</t>
         </is>
       </c>
     </row>
@@ -2628,7 +2628,7 @@
       </c>
       <c r="H44" s="15" t="inlineStr">
         <is>
-          <t>R: guía del MINSA de 2012 US$1,000; SignatureLex B/.1,500; la tarifa vigente no está publicada pese a la Ley 419 art. 79</t>
+          <t>R: guía del MINSA de 2012 US$1,000; SignatureLex B/.1,500; la tasa vigente no está publicada pese a la Ley 419 art. 79</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Segunda pasada de revisión: supuestos explícitos y archivo de investigación
- Plan: la fecha de la próxima LPU queda como estimación por el ciclo de la
  01-2026; el margen de Zywie (15%) queda como supuesto.
- Negociación y resumen en inglés: «equivalencia terapéutica» (bioequivalencia o
  bioexención, Res. 985 de 2025) en lugar de «estudios de bioequivalencia».
- DD: sin conteo fijo de afirmaciones.
- Excel: hoja de vida útil con la regla del pliego (ficha técnica; 18 meses si no
  la fija). Excel = motor en los cuatro casos.
- research/LEAME.md: qué es vigente (verificación del 9 de octubre) y qué es
  archivo de las rondas 1 y 2.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0135fezQES4kQref5cVQmNrQ
</commit_message>
<xml_diff>
--- a/outputs/Modelo_financiero.xlsx
+++ b/outputs/Modelo_financiero.xlsx
@@ -920,7 +920,7 @@
     <row r="1">
       <c r="B1" s="6" t="inlineStr">
         <is>
-          <t>Presupuesto de vida útil (regla de 18 meses al entregar)</t>
+          <t>Presupuesto de vida útil (pliego de la LPU: vencimiento de la ficha técnica; 18 meses si no lo fija)</t>
         </is>
       </c>
     </row>
@@ -937,7 +937,7 @@
     <row r="4">
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Vida útil mínima exigida al entregar (pliego de la LPU)</t>
+          <t>Vida útil exigida al entregar (18 meses si la ficha técnica no fija otra)</t>
         </is>
       </c>
       <c r="C4" s="46" t="n">
@@ -1473,7 +1473,7 @@
       </c>
       <c r="H11" s="15" t="inlineStr">
         <is>
-          <t>F: la LPU 01-2026 vence el 11-may-2027 y la siguiente se licitaría entre dic-2026 y feb-2027, antes de tener registros; la que sigue arrancaría hacia ago-2028 (mes 20). Optimista: la CSS prorroga y licita a inicios de 2028; pesimista: el calendario se corre 7 meses</t>
+          <t>F: la LPU 01-2026 vence el 11-may-2027; E: si se repite su ciclo, la siguiente se licita entre dic-2026 y feb-2027, antes de tener registros, y la que sigue arrancaría hacia ago-2028 (mes 20). Optimista: la CSS prorroga y licita a inicios de 2028; pesimista: el calendario se corre 7 meses</t>
         </is>
       </c>
     </row>

</xml_diff>